<commit_message>
Final hyperparameter tuning experiment done with SCAgent
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_groq_debateagent.xlsx
+++ b/orchestrator/results/aime24_groq_debateagent.xlsx
@@ -413,13 +413,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="n">
         <v>0</v>
       </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -430,6 +436,12 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -440,6 +452,12 @@
       <c r="B3" t="n">
         <v>0</v>
       </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -450,6 +468,12 @@
       <c r="B4" t="n">
         <v>0</v>
       </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -457,8 +481,20 @@
           <t>problems</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>1</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -468,7 +504,13 @@
         </is>
       </c>
       <c r="B6" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -478,7 +520,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0.23</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
@@ -490,6 +538,12 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
+      <c r="C8" t="n">
+        <v>56941</v>
+      </c>
+      <c r="D8" t="n">
+        <v>56941</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -500,6 +554,12 @@
       <c r="B9" t="n">
         <v>0</v>
       </c>
+      <c r="C9" t="n">
+        <v>0.00626351</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.00626351</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -510,6 +570,12 @@
       <c r="B10" t="n">
         <v>0</v>
       </c>
+      <c r="C10" t="n">
+        <v>17364</v>
+      </c>
+      <c r="D10" t="n">
+        <v>17364</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -520,6 +586,12 @@
       <c r="B11" t="n">
         <v>0</v>
       </c>
+      <c r="C11" t="n">
+        <v>0.00590376</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.00590376</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -528,7 +600,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1924</v>
+        <v>56941</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -538,7 +616,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.00021164</v>
+        <v>0.00626351</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -548,7 +632,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>837</v>
+        <v>17364</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -558,7 +648,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.00028458</v>
+        <v>0.00590376</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -570,6 +666,12 @@
       <c r="B16" t="n">
         <v>0</v>
       </c>
+      <c r="C16" t="n">
+        <v>14047</v>
+      </c>
+      <c r="D16" t="n">
+        <v>99248</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -580,6 +682,12 @@
       <c r="B17" t="n">
         <v>0</v>
       </c>
+      <c r="C17" t="n">
+        <v>0.00154517</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.01091728</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -590,6 +698,12 @@
       <c r="B18" t="n">
         <v>0</v>
       </c>
+      <c r="C18" t="n">
+        <v>55495</v>
+      </c>
+      <c r="D18" t="n">
+        <v>81222</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -600,6 +714,12 @@
       <c r="B19" t="n">
         <v>0</v>
       </c>
+      <c r="C19" t="n">
+        <v>0.0188683</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.02761548</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -608,7 +728,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2922</v>
+        <v>62378</v>
+      </c>
+      <c r="C20" t="n">
+        <v>118971</v>
+      </c>
+      <c r="D20" t="n">
+        <v>97280</v>
       </c>
     </row>
     <row r="21">
@@ -618,7 +744,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.00032142</v>
+        <v>0.00686158</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.01308681</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.0107008</v>
       </c>
     </row>
     <row r="22">
@@ -628,7 +760,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2287</v>
+        <v>65366</v>
+      </c>
+      <c r="C22" t="n">
+        <v>33167</v>
+      </c>
+      <c r="D22" t="n">
+        <v>31954</v>
       </c>
     </row>
     <row r="23">
@@ -638,7 +776,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.00077758</v>
+        <v>0.02222444</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.01127678</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.01086436</v>
       </c>
     </row>
     <row r="24">
@@ -650,6 +794,12 @@
       <c r="B24" t="n">
         <v>0</v>
       </c>
+      <c r="C24" t="n">
+        <v>30</v>
+      </c>
+      <c r="D24" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -658,7 +808,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>30</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -670,6 +826,12 @@
       <c r="B26" t="n">
         <v>0</v>
       </c>
+      <c r="C26" t="n">
+        <v>60</v>
+      </c>
+      <c r="D26" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -678,7 +840,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>90</v>
+      </c>
+      <c r="C27" t="n">
+        <v>90</v>
+      </c>
+      <c r="D27" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="28">
@@ -688,7 +856,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>36.46</v>
+        <v>364.6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>291.31</v>
+      </c>
+      <c r="D28" t="n">
+        <v>258.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>